<commit_message>
updated README with name
</commit_message>
<xml_diff>
--- a/student data.xlsx
+++ b/student data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AnudipCOA\Git-github_pratice\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D4FF4A4-9EF8-4E12-A7C7-20D82C6593A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F3EBE15-EDE7-4BC5-BEBB-6192908DFD95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3120" yWindow="3240" windowWidth="18000" windowHeight="9540" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,27 +25,27 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="7">
-  <si>
-    <t>sdfdfdf</t>
-  </si>
-  <si>
-    <t>dcf</t>
-  </si>
-  <si>
-    <t>frdds</t>
-  </si>
-  <si>
-    <t>fs</t>
-  </si>
-  <si>
-    <t>sa</t>
-  </si>
-  <si>
-    <t>asas</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t>d</t>
+  </si>
+  <si>
+    <t>sdsxfgschfs</t>
+  </si>
+  <si>
+    <t>sdd</t>
+  </si>
+  <si>
+    <t>xsdss</t>
+  </si>
+  <si>
+    <t>sxsxsx000xs</t>
+  </si>
+  <si>
+    <t>xssxsxs</t>
+  </si>
+  <si>
+    <t>xsxsx</t>
   </si>
 </sst>
 </file>
@@ -363,43 +363,38 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" t="s">
-        <v>4</v>
+      <c r="A2" t="s">
+        <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="E3" t="s">
-        <v>5</v>
+      <c r="A3" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="D4" t="s">
+      <c r="A4" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>5</v>
+      </c>
       <c r="B5" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="D6" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>